<commit_message>
Initial Googl Model and Updates
</commit_message>
<xml_diff>
--- a/Big 4 Capex vs OCF.xlsx
+++ b/Big 4 Capex vs OCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerem\OneDrive\Masaüstü\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D625FC4E-4EF3-4F59-B1B9-31143F49F9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8E058A-2385-477C-B20E-0D533F15C387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="804" windowWidth="23040" windowHeight="11760" xr2:uid="{DD181D79-B43F-4101-885F-595C61B85884}"/>
+    <workbookView minimized="1" xWindow="36" yWindow="12" windowWidth="23016" windowHeight="12336" xr2:uid="{DD181D79-B43F-4101-885F-595C61B85884}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Googl and MSFT Updates
</commit_message>
<xml_diff>
--- a/Big 4 Capex vs OCF.xlsx
+++ b/Big 4 Capex vs OCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerem\OneDrive\Masaüstü\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8E058A-2385-477C-B20E-0D533F15C387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E890913-5ED6-4048-BD36-ACF3EAB0B809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="36" yWindow="12" windowWidth="23016" windowHeight="12336" xr2:uid="{DD181D79-B43F-4101-885F-595C61B85884}"/>
+    <workbookView xWindow="20604" yWindow="468" windowWidth="32220" windowHeight="15948" xr2:uid="{DD181D79-B43F-4101-885F-595C61B85884}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -9701,7 +9701,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="8">
+  <wetp:taskpane dockstate="right" visibility="1" width="438" row="8">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>

</xml_diff>